<commit_message>
Redaktionsplan: Druckdaten-Check am 13.10. eingefügt, Termine 1 bis 3 korrigiert
Neuer Eintrag Nr. 25 füllt den freien Termin nach dem vorgezogenen Testpost,
übrige Termine unverändert. Import-Skript sortiert Einträge nach Datum.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bDdJteC7Rh81wY3gqmAnX
</commit_message>
<xml_diff>
--- a/plans/Redaktionsplan_Social_Media_Q4_2026.xlsx
+++ b/plans/Redaktionsplan_Social_Media_Q4_2026.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -158,7 +159,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -259,6 +260,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="17" min="1" max="2"/>
@@ -669,14 +671,14 @@
         <v>1</v>
       </c>
       <c r="B5" s="22" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="23" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Di</t>
+          <t>So</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -738,7 +740,7 @@
       </c>
       <c r="O5" s="22" t="inlineStr">
         <is>
-          <t>Entwurf</t>
+          <t>Gepostet</t>
         </is>
       </c>
     </row>
@@ -750,11 +752,11 @@
         <v>41</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="D6" s="22" t="inlineStr">
         <is>
-          <t>Do</t>
+          <t>Di</t>
         </is>
       </c>
       <c r="E6" s="22" t="inlineStr">
@@ -824,14 +826,14 @@
         <v>3</v>
       </c>
       <c r="B7" s="24" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="25" t="n">
-        <v>46308</v>
+        <v>46303</v>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>Di</t>
+          <t>Do</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
@@ -2515,6 +2517,111 @@
       </c>
       <c r="N28" s="22" t="n"/>
       <c r="O28" s="22" t="inlineStr">
+        <is>
+          <t>Entwurf</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" t="n">
+        <v>42</v>
+      </c>
+      <c r="C29" s="34" t="n">
+        <v>46308</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Di</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ratgeber</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Druckdaten-Check: fünf Punkte vor dem Upload</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Karussell (7 Slides: Titel, 5 Punkte, Abschluss)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>DRUCKDATEN? ERST PRÜFEN, DANN HOCHLADEN.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Druckdaten-Check: fünf Punkte vor dem Upload.
+Damit Ihr Motiv auf dem Stoff so wirkt wie geplant, lohnt sich ein kurzer Blick auf diese Punkte:
+1. Format passend zur Druckvorlage
+Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
+2. Bildauflösung mindestens 120 dpi
+Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
+3. Schriften in Pfade umwandeln
+So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
+4. Farbraum CMYK
+RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
+5. Überdrucken deaktivieren
+Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
+Keine Zeit für die Datenaufbereitung? Unser Grafikservice passt vorhandene Dateien an die Druckvorlage an.
+Alle Druckinformationen finden Sie auf zipperwalls.de</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Druckdaten-Check: fünf Punkte vor dem Upload.
+Damit Ihr Motiv auf dem Stoff so wirkt wie geplant, lohnt sich vor dem Hochladen ein kurzer Blick auf diese Punkte:
+1. Format passend zur Druckvorlage
+Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
+2. Bildauflösung mindestens 120 dpi
+Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
+3. Schriften in Pfade umwandeln
+So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
+4. Farbraum CMYK
+RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
+5. Überdrucken deaktivieren
+Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
+Keine Zeit für die Datenaufbereitung? Unser Grafikservice passt vorhandene Dateien an die Druckvorlage an.
+Alle Druckinformationen: https://www.zipperwalls.de/kundenservice/druckinformationen/</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Der häufigste Engpass vor der Messe sind nicht die Systeme, sondern die Druckdaten.
+Fünf Punkte, die wir vor jedem Upload empfehlen:
+1. Format passend zur Druckvorlage
+Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
+2. Bildauflösung mindestens 120 dpi
+Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
+3. Schriften in Pfade umwandeln
+So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
+4. Farbraum CMYK
+RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
+5. Überdrucken deaktivieren
+Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
+Wer diese fünf Punkte prüft, spart Korrekturschleifen und Zeit vor dem Messetermin. Alle Druckinformationen: https://www.zipperwalls.de/kundenservice/druckinformationen/</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>#druckdaten #textildruck #messewand #messetipp #zipperwalls</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Neu eingefügt am 04.10.2026 für den freien Termin am 13.10. Fakten aus den Zipperwalls-Druckvorgaben. Link zu den Druckinformationen vor Veröffentlichung prüfen.</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>Entwurf</t>
         </is>

</xml_diff>

<commit_message>
Redaktionsplan: Nr. 25 neues Thema Hinter den Kulissen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bDdJteC7Rh81wY3gqmAnX
</commit_message>
<xml_diff>
--- a/plans/Redaktionsplan_Social_Media_Q4_2026.xlsx
+++ b/plans/Redaktionsplan_Social_Media_Q4_2026.xlsx
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -2523,105 +2522,95 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="17" t="n">
         <v>42</v>
       </c>
       <c r="C29" s="34" t="n">
         <v>46308</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>Di</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Ratgeber</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Druckdaten-Check: fünf Punkte vor dem Upload</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>Karussell (7 Slides: Titel, 5 Punkte, Abschluss)</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>DRUCKDATEN? ERST PRÜFEN, DANN HOCHLADEN.</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Druckdaten-Check: fünf Punkte vor dem Upload.
-Damit Ihr Motiv auf dem Stoff so wirkt wie geplant, lohnt sich ein kurzer Blick auf diese Punkte:
-1. Format passend zur Druckvorlage
-Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
-2. Bildauflösung mindestens 120 dpi
-Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
-3. Schriften in Pfade umwandeln
-So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
-4. Farbraum CMYK
-RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
-5. Überdrucken deaktivieren
-Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
-Keine Zeit für die Datenaufbereitung? Unser Grafikservice passt vorhandene Dateien an die Druckvorlage an.
-Alle Druckinformationen finden Sie auf zipperwalls.de</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Druckdaten-Check: fünf Punkte vor dem Upload.
-Damit Ihr Motiv auf dem Stoff so wirkt wie geplant, lohnt sich vor dem Hochladen ein kurzer Blick auf diese Punkte:
-1. Format passend zur Druckvorlage
-Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
-2. Bildauflösung mindestens 120 dpi
-Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
-3. Schriften in Pfade umwandeln
-So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
-4. Farbraum CMYK
-RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
-5. Überdrucken deaktivieren
-Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
-Keine Zeit für die Datenaufbereitung? Unser Grafikservice passt vorhandene Dateien an die Druckvorlage an.
-Alle Druckinformationen: https://www.zipperwalls.de/kundenservice/druckinformationen/</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Der häufigste Engpass vor der Messe sind nicht die Systeme, sondern die Druckdaten.
-Fünf Punkte, die wir vor jedem Upload empfehlen:
-1. Format passend zur Druckvorlage
-Legen Sie Ihr Motiv direkt in der Druckvorlage des jeweiligen Produkts an. So stimmen Maße und Beschnitt.
-2. Bildauflösung mindestens 120 dpi
-Gemessen bei 100 % Skalierung, also in Endgröße. Darunter wirken Fotos auf großen Flächen schnell unscharf.
-3. Schriften in Pfade umwandeln
-So wird jede Schrift genau so gedruckt, wie Sie sie gestaltet haben, auch wenn sie uns nicht vorliegt.
-4. Farbraum CMYK
-RGB-Daten werden für den Druck automatisch umgewandelt. Dabei können sich Farben leicht verschieben. Mit CMYK-Daten haben Sie das Ergebnis besser im Griff.
-5. Überdrucken deaktivieren
-Ist Überdrucken aktiv, können Elemente im Druck verschwinden oder Farben sich ungewollt mischen.
-Wer diese fünf Punkte prüft, spart Korrekturschleifen und Zeit vor dem Messetermin. Alle Druckinformationen: https://www.zipperwalls.de/kundenservice/druckinformationen/</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>#druckdaten #textildruck #messewand #messetipp #zipperwalls</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>Neu eingefügt am 04.10.2026 für den freien Termin am 13.10. Fakten aus den Zipperwalls-Druckvorgaben. Link zu den Druckinformationen vor Veröffentlichung prüfen.</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>Hinter den Kulissen</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
+        <is>
+          <t>Hinter den Kulissen: So läuft Ihre Bestellung ab</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Karussell (6 Slides: Titel, 4 Schritte, Abschluss)</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>VON DER IDEE ZUR MESSEWAND.</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>So läuft Ihre Bestellung bei Zipperwalls ab.
+Von der ersten Idee bis zur fertigen Messewand in vier Schritten:
+1. Produkt konfigurieren
+Im Shop wählen Sie Größe, ein- oder beidseitigen Druck und die Transportlösung, zum Beispiel Tasche oder Trolley. Bei Fragen zu Größe oder Ausstattung beraten wir Sie persönlich, Mo bis Fr von 8 bis 17 Uhr.
+2. Druckdaten anlegen
+Sie legen Ihr Motiv in der Druckvorlage des jeweiligen Produkts an. Keine eigenen Daten? Unser Grafikservice gestaltet Ihr Layout oder passt vorhandene Dateien an.
+3. Daten prüfen
+Vor der Produktion werden Ihre Druckdaten geprüft, zum Beispiel auf Auflösung, Schriften und Farbraum. So fallen Fehler auf, bevor gedruckt wird.
+4. Produktion und Versand
+Ihr Stoffdruck entsteht im Sublimationsverfahren, B1-zertifiziert und bei 30 °C waschbar. Danach geht alles fertig verpackt auf den Weg zu Ihnen.
+Fragen zu Ihrem Projekt? Wir sind persönlich für Sie da.</t>
+        </is>
+      </c>
+      <c r="J29" s="17" t="inlineStr">
+        <is>
+          <t>Von der Idee zur fertigen Messewand: So läuft Ihre Bestellung bei Zipperwalls ab.
+1. Produkt konfigurieren
+Im Shop wählen Sie Größe, ein- oder beidseitigen Druck und die Transportlösung, zum Beispiel Tasche oder Trolley. Bei Fragen zu Größe oder Ausstattung beraten wir Sie persönlich, Mo bis Fr von 8 bis 17 Uhr.
+2. Druckdaten anlegen
+Sie legen Ihr Motiv in der Druckvorlage des jeweiligen Produkts an. Keine eigenen Daten? Unser Grafikservice gestaltet Ihr Layout oder passt vorhandene Dateien an.
+3. Daten prüfen
+Vor der Produktion werden Ihre Druckdaten geprüft, zum Beispiel auf Auflösung, Schriften und Farbraum. So fallen Fehler auf, bevor gedruckt wird.
+4. Produktion und Versand
+Ihr Stoffdruck entsteht im Sublimationsverfahren, B1-zertifiziert und bei 30 °C waschbar. Danach geht alles fertig verpackt auf den Weg zu Ihnen.
+Fragen zu Ihrem Projekt? Sie erreichen uns Mo bis Fr von 8 bis 17 Uhr unter +49 7276 4049970.</t>
+        </is>
+      </c>
+      <c r="K29" s="17" t="inlineStr">
+        <is>
+          <t>Ein Messeauftritt beginnt lange vor dem Aufbau. So läuft eine Bestellung bei Zipperwalls ab:
+1. Produkt konfigurieren
+Im Shop wählen Sie Größe, ein- oder beidseitigen Druck und die Transportlösung, zum Beispiel Tasche oder Trolley. Bei Fragen zu Größe oder Ausstattung beraten wir Sie persönlich, Mo bis Fr von 8 bis 17 Uhr.
+2. Druckdaten anlegen
+Sie legen Ihr Motiv in der Druckvorlage des jeweiligen Produkts an. Keine eigenen Daten? Unser Grafikservice gestaltet Ihr Layout oder passt vorhandene Dateien an.
+3. Daten prüfen
+Vor der Produktion werden Ihre Druckdaten geprüft, zum Beispiel auf Auflösung, Schriften und Farbraum. So fallen Fehler auf, bevor gedruckt wird.
+4. Produktion und Versand
+Ihr Stoffdruck entsteht im Sublimationsverfahren, B1-zertifiziert und bei 30 °C waschbar. Danach geht alles fertig verpackt auf den Weg zu Ihnen.
+So wissen Sie bei jedem Schritt, woran Sie sind. Fragen zu Ihrem Projekt beantworten wir gern persönlich.</t>
+        </is>
+      </c>
+      <c r="L29" s="17" t="inlineStr">
+        <is>
+          <t>#hinterdenkulissen #messewand #textildruck #messestand #zipperwalls</t>
+        </is>
+      </c>
+      <c r="M29" s="17" t="inlineStr"/>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>Neu eingefügt am 04.10.2026 für den freien Termin am 13.10. (ersetzt den Druckdaten-Check, der sich mit Newsletter Nr. 4 doppelte). Vor Veröffentlichung prüfen: Ablauf des Datenchecks und Versand so korrekt beschrieben?</t>
+        </is>
+      </c>
+      <c r="O29" s="17" t="inlineStr">
         <is>
           <t>Entwurf</t>
         </is>

</xml_diff>